<commit_message>
Add Yuezheng Ling library and expand presets
</commit_message>
<xml_diff>
--- a/outputs/vcpedia-crawl/luotianyi-legend-songs-review2.xlsx
+++ b/outputs/vcpedia-crawl/luotianyi-legend-songs-review2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AProjects\luo-yi-ba\outputs\vcpedia-crawl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9883956-3BEA-4320-9D4F-73C520698528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB8841C-F97C-488D-8451-DF16F100F088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="曲目数据" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2872" uniqueCount="1117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2872" uniqueCount="1118">
   <si>
     <t>序号</t>
   </si>
@@ -3374,6 +3374,10 @@
   </si>
   <si>
     <t>歌曲页面 URL</t>
+    <phoneticPr fontId="10" type="noConversion"/>
+  </si>
+  <si>
+    <t>拜年/贺岁纪曲目</t>
     <phoneticPr fontId="10" type="noConversion"/>
   </si>
 </sst>
@@ -3783,14 +3787,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="SongReviewTable" displayName="SongReviewTable" ref="A1:J220" totalsRowShown="0">
-  <autoFilter ref="A1:J220" xr:uid="{00000000-0009-0000-0100-000003000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="VOCALOID；ACE Studio；X Studio"/>
-        <filter val="VOCALOID；Synthesizer V"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:J220" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="序号"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="曲名"/>
@@ -4065,7 +4062,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="2" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A2" s="14">
         <v>1</v>
       </c>
@@ -4097,7 +4094,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="3" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A3" s="19">
         <v>2</v>
       </c>
@@ -4129,7 +4126,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="4" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A4" s="19">
         <v>3</v>
       </c>
@@ -4161,7 +4158,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="5" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A5" s="19">
         <v>4</v>
       </c>
@@ -4193,7 +4190,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="6" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A6" s="19">
         <v>5</v>
       </c>
@@ -4225,7 +4222,7 @@
         <v>889</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="7" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A7" s="19">
         <v>6</v>
       </c>
@@ -4257,7 +4254,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="8" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A8" s="19">
         <v>7</v>
       </c>
@@ -4289,7 +4286,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="9" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A9" s="19">
         <v>8</v>
       </c>
@@ -4321,7 +4318,7 @@
         <v>892</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="10" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A10" s="19">
         <v>9</v>
       </c>
@@ -4353,7 +4350,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="11" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A11" s="19">
         <v>10</v>
       </c>
@@ -4385,7 +4382,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="12" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A12" s="19">
         <v>11</v>
       </c>
@@ -4417,7 +4414,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="13" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A13" s="19">
         <v>12</v>
       </c>
@@ -4449,7 +4446,7 @@
         <v>896</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="14" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A14" s="19">
         <v>13</v>
       </c>
@@ -4481,7 +4478,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="15" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A15" s="19">
         <v>14</v>
       </c>
@@ -4513,7 +4510,7 @@
         <v>898</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="16" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A16" s="19">
         <v>15</v>
       </c>
@@ -4545,7 +4542,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="17" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A17" s="19">
         <v>16</v>
       </c>
@@ -4577,7 +4574,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="18" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A18" s="19">
         <v>17</v>
       </c>
@@ -4609,7 +4606,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="19" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A19" s="19">
         <v>18</v>
       </c>
@@ -4641,7 +4638,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="20" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A20" s="19">
         <v>19</v>
       </c>
@@ -4673,7 +4670,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="21" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A21" s="19">
         <v>20</v>
       </c>
@@ -4705,7 +4702,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="22" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A22" s="19">
         <v>21</v>
       </c>
@@ -4737,7 +4734,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="23" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A23" s="19">
         <v>22</v>
       </c>
@@ -4769,7 +4766,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="24" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A24" s="19">
         <v>23</v>
       </c>
@@ -4792,7 +4789,7 @@
         <v>6</v>
       </c>
       <c r="H24" s="23" t="s">
-        <v>76</v>
+        <v>1117</v>
       </c>
       <c r="I24" s="26" t="s">
         <v>77</v>
@@ -4801,7 +4798,7 @@
         <v>907</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="25" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A25" s="19">
         <v>24</v>
       </c>
@@ -4833,7 +4830,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="26" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A26" s="19">
         <v>25</v>
       </c>
@@ -4865,7 +4862,7 @@
         <v>909</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="27" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A27" s="19">
         <v>26</v>
       </c>
@@ -4897,7 +4894,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="28" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A28" s="19">
         <v>27</v>
       </c>
@@ -4929,7 +4926,7 @@
         <v>911</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="29" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A29" s="19">
         <v>28</v>
       </c>
@@ -4961,7 +4958,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="30" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A30" s="19">
         <v>29</v>
       </c>
@@ -4993,7 +4990,7 @@
         <v>913</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="31" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A31" s="19">
         <v>30</v>
       </c>
@@ -5025,7 +5022,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="32" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A32" s="19">
         <v>31</v>
       </c>
@@ -5057,7 +5054,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="33" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A33" s="19">
         <v>32</v>
       </c>
@@ -5089,7 +5086,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="34" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A34" s="19">
         <v>33</v>
       </c>
@@ -5121,7 +5118,7 @@
         <v>917</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="35" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A35" s="19">
         <v>34</v>
       </c>
@@ -5153,7 +5150,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="36" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A36" s="19">
         <v>35</v>
       </c>
@@ -5185,7 +5182,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="37" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A37" s="19">
         <v>36</v>
       </c>
@@ -5217,7 +5214,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="38" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A38" s="19">
         <v>37</v>
       </c>
@@ -5249,7 +5246,7 @@
         <v>921</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="39" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A39" s="19">
         <v>38</v>
       </c>
@@ -5281,7 +5278,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="40" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A40" s="19">
         <v>39</v>
       </c>
@@ -5313,7 +5310,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="41" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A41" s="19">
         <v>40</v>
       </c>
@@ -5345,7 +5342,7 @@
         <v>924</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="42" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A42" s="19">
         <v>41</v>
       </c>
@@ -5377,7 +5374,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="43" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A43" s="19">
         <v>42</v>
       </c>
@@ -5409,7 +5406,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="44" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A44" s="19">
         <v>43</v>
       </c>
@@ -5441,7 +5438,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="45" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A45" s="19">
         <v>44</v>
       </c>
@@ -5473,7 +5470,7 @@
         <v>928</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="46" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A46" s="19">
         <v>45</v>
       </c>
@@ -5505,7 +5502,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="47" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A47" s="19">
         <v>46</v>
       </c>
@@ -5537,7 +5534,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="48" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A48" s="19">
         <v>47</v>
       </c>
@@ -5569,7 +5566,7 @@
         <v>931</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="49" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A49" s="19">
         <v>48</v>
       </c>
@@ -5601,7 +5598,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="50" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A50" s="19">
         <v>49</v>
       </c>
@@ -5633,7 +5630,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="51" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A51" s="19">
         <v>50</v>
       </c>
@@ -5665,7 +5662,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="52" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A52" s="19">
         <v>51</v>
       </c>
@@ -5697,7 +5694,7 @@
         <v>935</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="53" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A53" s="19">
         <v>52</v>
       </c>
@@ -5729,7 +5726,7 @@
         <v>936</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="54" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A54" s="19">
         <v>53</v>
       </c>
@@ -5761,7 +5758,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="55" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A55" s="19">
         <v>54</v>
       </c>
@@ -5793,7 +5790,7 @@
         <v>938</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="56" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A56" s="19">
         <v>55</v>
       </c>
@@ -5825,7 +5822,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="57" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A57" s="19">
         <v>56</v>
       </c>
@@ -5857,7 +5854,7 @@
         <v>940</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="58" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A58" s="19">
         <v>57</v>
       </c>
@@ -5889,7 +5886,7 @@
         <v>941</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="59" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A59" s="19">
         <v>58</v>
       </c>
@@ -5921,7 +5918,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="60" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A60" s="19">
         <v>59</v>
       </c>
@@ -5953,7 +5950,7 @@
         <v>943</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="61" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A61" s="19">
         <v>60</v>
       </c>
@@ -5985,7 +5982,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="62" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A62" s="19">
         <v>61</v>
       </c>
@@ -6017,7 +6014,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="63" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A63" s="19">
         <v>62</v>
       </c>
@@ -6049,7 +6046,7 @@
         <v>946</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="64" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A64" s="19">
         <v>63</v>
       </c>
@@ -6081,7 +6078,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="65" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A65" s="19">
         <v>64</v>
       </c>
@@ -6113,7 +6110,7 @@
         <v>948</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="66" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A66" s="19">
         <v>65</v>
       </c>
@@ -6145,7 +6142,7 @@
         <v>949</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="67" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A67" s="19">
         <v>66</v>
       </c>
@@ -6177,7 +6174,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="68" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A68" s="19">
         <v>67</v>
       </c>
@@ -6209,7 +6206,7 @@
         <v>951</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="69" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A69" s="19">
         <v>68</v>
       </c>
@@ -6241,7 +6238,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="70" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A70" s="19">
         <v>69</v>
       </c>
@@ -6273,7 +6270,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="71" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A71" s="19">
         <v>70</v>
       </c>
@@ -6305,7 +6302,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="72" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A72" s="19">
         <v>71</v>
       </c>
@@ -6337,7 +6334,7 @@
         <v>955</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="73" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A73" s="19">
         <v>72</v>
       </c>
@@ -6369,7 +6366,7 @@
         <v>956</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="74" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A74" s="19">
         <v>73</v>
       </c>
@@ -6401,7 +6398,7 @@
         <v>957</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="75" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A75" s="19">
         <v>74</v>
       </c>
@@ -6433,7 +6430,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="76" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="76" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A76" s="19">
         <v>75</v>
       </c>
@@ -6465,7 +6462,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="77" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A77" s="19">
         <v>76</v>
       </c>
@@ -6497,7 +6494,7 @@
         <v>960</v>
       </c>
     </row>
-    <row r="78" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="78" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A78" s="19">
         <v>77</v>
       </c>
@@ -6529,7 +6526,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="79" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="79" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A79" s="19">
         <v>78</v>
       </c>
@@ -6561,7 +6558,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="80" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="80" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A80" s="19">
         <v>79</v>
       </c>
@@ -6593,7 +6590,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="81" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="81" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A81" s="19">
         <v>80</v>
       </c>
@@ -6625,7 +6622,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="82" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="82" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A82" s="19">
         <v>81</v>
       </c>
@@ -6657,7 +6654,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="83" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="83" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A83" s="19">
         <v>82</v>
       </c>
@@ -6689,7 +6686,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="84" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="84" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A84" s="19">
         <v>83</v>
       </c>
@@ -6721,7 +6718,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="85" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="85" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A85" s="19">
         <v>84</v>
       </c>
@@ -6753,7 +6750,7 @@
         <v>968</v>
       </c>
     </row>
-    <row r="86" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="86" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A86" s="19">
         <v>85</v>
       </c>
@@ -6785,7 +6782,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="87" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="87" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A87" s="19">
         <v>86</v>
       </c>
@@ -6817,7 +6814,7 @@
         <v>970</v>
       </c>
     </row>
-    <row r="88" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="88" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A88" s="19">
         <v>87</v>
       </c>
@@ -6849,7 +6846,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="89" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="89" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A89" s="19">
         <v>88</v>
       </c>
@@ -6881,7 +6878,7 @@
         <v>972</v>
       </c>
     </row>
-    <row r="90" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="90" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A90" s="19">
         <v>89</v>
       </c>
@@ -6913,7 +6910,7 @@
         <v>973</v>
       </c>
     </row>
-    <row r="91" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="91" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A91" s="19">
         <v>90</v>
       </c>
@@ -6945,7 +6942,7 @@
         <v>974</v>
       </c>
     </row>
-    <row r="92" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="92" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A92" s="19">
         <v>91</v>
       </c>
@@ -6977,7 +6974,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="93" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="93" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A93" s="19">
         <v>92</v>
       </c>
@@ -7009,7 +7006,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="94" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="94" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A94" s="19">
         <v>93</v>
       </c>
@@ -7041,7 +7038,7 @@
         <v>977</v>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="95" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A95" s="19">
         <v>94</v>
       </c>
@@ -7073,7 +7070,7 @@
         <v>978</v>
       </c>
     </row>
-    <row r="96" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="96" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A96" s="19">
         <v>95</v>
       </c>
@@ -7105,7 +7102,7 @@
         <v>979</v>
       </c>
     </row>
-    <row r="97" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="97" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A97" s="19">
         <v>96</v>
       </c>
@@ -7137,7 +7134,7 @@
         <v>980</v>
       </c>
     </row>
-    <row r="98" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="98" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A98" s="19">
         <v>97</v>
       </c>
@@ -7169,7 +7166,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="99" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="99" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A99" s="19">
         <v>98</v>
       </c>
@@ -7201,7 +7198,7 @@
         <v>982</v>
       </c>
     </row>
-    <row r="100" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="100" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A100" s="19">
         <v>99</v>
       </c>
@@ -7233,7 +7230,7 @@
         <v>983</v>
       </c>
     </row>
-    <row r="101" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="101" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A101" s="19">
         <v>100</v>
       </c>
@@ -7265,7 +7262,7 @@
         <v>984</v>
       </c>
     </row>
-    <row r="102" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="102" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A102" s="19">
         <v>101</v>
       </c>
@@ -7297,7 +7294,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="103" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="103" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A103" s="19">
         <v>102</v>
       </c>
@@ -7329,7 +7326,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="104" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="104" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A104" s="19">
         <v>103</v>
       </c>
@@ -7361,7 +7358,7 @@
         <v>987</v>
       </c>
     </row>
-    <row r="105" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="105" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A105" s="19">
         <v>104</v>
       </c>
@@ -7393,7 +7390,7 @@
         <v>988</v>
       </c>
     </row>
-    <row r="106" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="106" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A106" s="19">
         <v>105</v>
       </c>
@@ -7425,7 +7422,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="107" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="107" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A107" s="19">
         <v>106</v>
       </c>
@@ -7457,7 +7454,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="108" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="108" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A108" s="19">
         <v>107</v>
       </c>
@@ -7489,7 +7486,7 @@
         <v>991</v>
       </c>
     </row>
-    <row r="109" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="109" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A109" s="19">
         <v>108</v>
       </c>
@@ -7521,7 +7518,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="110" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="110" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A110" s="19">
         <v>109</v>
       </c>
@@ -7553,7 +7550,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="111" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="111" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A111" s="19">
         <v>110</v>
       </c>
@@ -7585,7 +7582,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="112" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="112" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A112" s="19">
         <v>111</v>
       </c>
@@ -7617,7 +7614,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="113" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="113" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A113" s="19">
         <v>112</v>
       </c>
@@ -7649,7 +7646,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="114" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="114" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A114" s="19">
         <v>113</v>
       </c>
@@ -7681,7 +7678,7 @@
         <v>997</v>
       </c>
     </row>
-    <row r="115" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="115" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A115" s="19">
         <v>114</v>
       </c>
@@ -7713,7 +7710,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="116" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="116" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A116" s="19">
         <v>115</v>
       </c>
@@ -7745,7 +7742,7 @@
         <v>999</v>
       </c>
     </row>
-    <row r="117" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="117" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A117" s="19">
         <v>116</v>
       </c>
@@ -7777,7 +7774,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="118" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="118" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A118" s="19">
         <v>117</v>
       </c>
@@ -7809,7 +7806,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="119" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="119" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A119" s="19">
         <v>118</v>
       </c>
@@ -7841,7 +7838,7 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="120" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="120" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A120" s="19">
         <v>119</v>
       </c>
@@ -7873,7 +7870,7 @@
         <v>1003</v>
       </c>
     </row>
-    <row r="121" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="121" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A121" s="19">
         <v>120</v>
       </c>
@@ -7905,7 +7902,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="122" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="122" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A122" s="19">
         <v>121</v>
       </c>
@@ -7937,7 +7934,7 @@
         <v>1005</v>
       </c>
     </row>
-    <row r="123" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="123" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A123" s="19">
         <v>122</v>
       </c>
@@ -7969,7 +7966,7 @@
         <v>1006</v>
       </c>
     </row>
-    <row r="124" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="124" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A124" s="19">
         <v>123</v>
       </c>
@@ -8001,7 +7998,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="125" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="125" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A125" s="19">
         <v>124</v>
       </c>
@@ -8033,7 +8030,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="126" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="126" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A126" s="19">
         <v>125</v>
       </c>
@@ -8097,7 +8094,7 @@
         <v>1010</v>
       </c>
     </row>
-    <row r="128" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="128" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A128" s="19">
         <v>127</v>
       </c>
@@ -8129,7 +8126,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="129" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="129" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A129" s="19">
         <v>128</v>
       </c>
@@ -8161,7 +8158,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="130" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="130" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A130" s="19">
         <v>129</v>
       </c>
@@ -8193,7 +8190,7 @@
         <v>1013</v>
       </c>
     </row>
-    <row r="131" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="131" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A131" s="19">
         <v>130</v>
       </c>
@@ -8225,7 +8222,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="132" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="132" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A132" s="19">
         <v>131</v>
       </c>
@@ -8257,7 +8254,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="133" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="133" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A133" s="19">
         <v>132</v>
       </c>
@@ -8289,7 +8286,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="134" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="134" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A134" s="19">
         <v>133</v>
       </c>
@@ -8321,7 +8318,7 @@
         <v>1017</v>
       </c>
     </row>
-    <row r="135" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="135" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A135" s="19">
         <v>134</v>
       </c>
@@ -8353,7 +8350,7 @@
         <v>1018</v>
       </c>
     </row>
-    <row r="136" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="136" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A136" s="19">
         <v>135</v>
       </c>
@@ -8385,7 +8382,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="137" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="137" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A137" s="19">
         <v>136</v>
       </c>
@@ -8417,7 +8414,7 @@
         <v>1020</v>
       </c>
     </row>
-    <row r="138" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="138" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A138" s="19">
         <v>137</v>
       </c>
@@ -8449,7 +8446,7 @@
         <v>1021</v>
       </c>
     </row>
-    <row r="139" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="139" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A139" s="19">
         <v>138</v>
       </c>
@@ -8481,7 +8478,7 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="140" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="140" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A140" s="19">
         <v>139</v>
       </c>
@@ -8513,7 +8510,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="141" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="141" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A141" s="19">
         <v>140</v>
       </c>
@@ -8545,7 +8542,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="142" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="142" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A142" s="19">
         <v>141</v>
       </c>
@@ -8577,7 +8574,7 @@
         <v>1025</v>
       </c>
     </row>
-    <row r="143" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="143" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A143" s="19">
         <v>142</v>
       </c>
@@ -8609,7 +8606,7 @@
         <v>1026</v>
       </c>
     </row>
-    <row r="144" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="144" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A144" s="19">
         <v>143</v>
       </c>
@@ -8641,7 +8638,7 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="145" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="145" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A145" s="19">
         <v>144</v>
       </c>
@@ -8673,7 +8670,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="146" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="146" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A146" s="19">
         <v>145</v>
       </c>
@@ -8705,7 +8702,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="147" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="147" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A147" s="19">
         <v>146</v>
       </c>
@@ -8737,7 +8734,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="148" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="148" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A148" s="19">
         <v>147</v>
       </c>
@@ -8769,7 +8766,7 @@
         <v>1031</v>
       </c>
     </row>
-    <row r="149" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="149" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A149" s="19">
         <v>148</v>
       </c>
@@ -8801,7 +8798,7 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="150" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="150" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A150" s="19">
         <v>149</v>
       </c>
@@ -8833,7 +8830,7 @@
         <v>1033</v>
       </c>
     </row>
-    <row r="151" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="151" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A151" s="19">
         <v>150</v>
       </c>
@@ -8865,7 +8862,7 @@
         <v>1034</v>
       </c>
     </row>
-    <row r="152" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="152" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A152" s="19">
         <v>151</v>
       </c>
@@ -8897,7 +8894,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="153" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="153" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A153" s="19">
         <v>152</v>
       </c>
@@ -8929,7 +8926,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="154" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="154" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A154" s="19">
         <v>153</v>
       </c>
@@ -8961,7 +8958,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="155" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="155" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A155" s="19">
         <v>154</v>
       </c>
@@ -8993,7 +8990,7 @@
         <v>1038</v>
       </c>
     </row>
-    <row r="156" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="156" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A156" s="19">
         <v>155</v>
       </c>
@@ -9025,7 +9022,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="157" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="157" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A157" s="19">
         <v>156</v>
       </c>
@@ -9057,7 +9054,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="158" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="158" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A158" s="19">
         <v>157</v>
       </c>
@@ -9089,7 +9086,7 @@
         <v>1041</v>
       </c>
     </row>
-    <row r="159" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="159" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A159" s="19">
         <v>158</v>
       </c>
@@ -9121,7 +9118,7 @@
         <v>1042</v>
       </c>
     </row>
-    <row r="160" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="160" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A160" s="19">
         <v>159</v>
       </c>
@@ -9153,7 +9150,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="161" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="161" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A161" s="19">
         <v>160</v>
       </c>
@@ -9185,7 +9182,7 @@
         <v>1044</v>
       </c>
     </row>
-    <row r="162" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="162" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A162" s="19">
         <v>161</v>
       </c>
@@ -9217,7 +9214,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="163" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="163" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A163" s="19">
         <v>162</v>
       </c>
@@ -9249,7 +9246,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="164" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="164" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A164" s="19">
         <v>163</v>
       </c>
@@ -9281,7 +9278,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="165" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="165" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A165" s="19">
         <v>164</v>
       </c>
@@ -9313,7 +9310,7 @@
         <v>1048</v>
       </c>
     </row>
-    <row r="166" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="166" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A166" s="19">
         <v>165</v>
       </c>
@@ -9345,7 +9342,7 @@
         <v>1049</v>
       </c>
     </row>
-    <row r="167" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="167" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A167" s="19">
         <v>166</v>
       </c>
@@ -9377,7 +9374,7 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="168" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="168" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A168" s="19">
         <v>167</v>
       </c>
@@ -9409,7 +9406,7 @@
         <v>1051</v>
       </c>
     </row>
-    <row r="169" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="169" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A169" s="19">
         <v>168</v>
       </c>
@@ -9441,7 +9438,7 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="170" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="170" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A170" s="19">
         <v>169</v>
       </c>
@@ -9473,7 +9470,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="171" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="171" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A171" s="19">
         <v>170</v>
       </c>
@@ -9505,7 +9502,7 @@
         <v>1054</v>
       </c>
     </row>
-    <row r="172" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="172" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A172" s="19">
         <v>171</v>
       </c>
@@ -9537,7 +9534,7 @@
         <v>1055</v>
       </c>
     </row>
-    <row r="173" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="173" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A173" s="19">
         <v>172</v>
       </c>
@@ -9569,7 +9566,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="174" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="174" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A174" s="19">
         <v>173</v>
       </c>
@@ -9601,7 +9598,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="175" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="175" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A175" s="19">
         <v>174</v>
       </c>
@@ -9633,7 +9630,7 @@
         <v>1058</v>
       </c>
     </row>
-    <row r="176" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="176" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A176" s="19">
         <v>175</v>
       </c>
@@ -9665,7 +9662,7 @@
         <v>1059</v>
       </c>
     </row>
-    <row r="177" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="177" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A177" s="19">
         <v>176</v>
       </c>
@@ -9697,7 +9694,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="178" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="178" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A178" s="19">
         <v>177</v>
       </c>
@@ -9729,7 +9726,7 @@
         <v>1061</v>
       </c>
     </row>
-    <row r="179" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="179" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A179" s="19">
         <v>178</v>
       </c>
@@ -9793,7 +9790,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="181" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="181" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A181" s="19">
         <v>180</v>
       </c>
@@ -9825,7 +9822,7 @@
         <v>1064</v>
       </c>
     </row>
-    <row r="182" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="182" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A182" s="19">
         <v>181</v>
       </c>
@@ -9857,7 +9854,7 @@
         <v>1065</v>
       </c>
     </row>
-    <row r="183" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="183" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A183" s="19">
         <v>182</v>
       </c>
@@ -9889,7 +9886,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="184" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="184" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A184" s="19">
         <v>183</v>
       </c>
@@ -9921,7 +9918,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="185" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="185" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A185" s="19">
         <v>184</v>
       </c>
@@ -9953,7 +9950,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="186" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="186" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A186" s="19">
         <v>185</v>
       </c>
@@ -9985,7 +9982,7 @@
         <v>1069</v>
       </c>
     </row>
-    <row r="187" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="187" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A187" s="19">
         <v>186</v>
       </c>
@@ -10017,7 +10014,7 @@
         <v>1070</v>
       </c>
     </row>
-    <row r="188" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="188" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A188" s="19">
         <v>187</v>
       </c>
@@ -10049,7 +10046,7 @@
         <v>1071</v>
       </c>
     </row>
-    <row r="189" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="189" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A189" s="19">
         <v>188</v>
       </c>
@@ -10081,7 +10078,7 @@
         <v>1072</v>
       </c>
     </row>
-    <row r="190" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="190" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A190" s="19">
         <v>189</v>
       </c>
@@ -10113,7 +10110,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="191" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="191" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A191" s="19">
         <v>190</v>
       </c>
@@ -10145,7 +10142,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="192" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="192" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A192" s="19">
         <v>191</v>
       </c>
@@ -10177,7 +10174,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="193" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="193" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A193" s="19">
         <v>192</v>
       </c>
@@ -10209,7 +10206,7 @@
         <v>1076</v>
       </c>
     </row>
-    <row r="194" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="194" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A194" s="19">
         <v>193</v>
       </c>
@@ -10241,7 +10238,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="195" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="195" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A195" s="19">
         <v>194</v>
       </c>
@@ -10273,7 +10270,7 @@
         <v>1078</v>
       </c>
     </row>
-    <row r="196" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="196" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A196" s="19">
         <v>195</v>
       </c>
@@ -10305,7 +10302,7 @@
         <v>1079</v>
       </c>
     </row>
-    <row r="197" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="197" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A197" s="19">
         <v>196</v>
       </c>
@@ -10337,7 +10334,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="198" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="198" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A198" s="19">
         <v>197</v>
       </c>
@@ -10369,7 +10366,7 @@
         <v>1081</v>
       </c>
     </row>
-    <row r="199" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="199" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A199" s="19">
         <v>198</v>
       </c>
@@ -10401,7 +10398,7 @@
         <v>1082</v>
       </c>
     </row>
-    <row r="200" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="200" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A200" s="19">
         <v>199</v>
       </c>
@@ -10433,7 +10430,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="201" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="201" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A201" s="19">
         <v>200</v>
       </c>
@@ -10465,7 +10462,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="202" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="202" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A202" s="19">
         <v>201</v>
       </c>
@@ -10497,7 +10494,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="203" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="203" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A203" s="19">
         <v>202</v>
       </c>
@@ -10529,7 +10526,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="204" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="204" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A204" s="19">
         <v>203</v>
       </c>
@@ -10561,7 +10558,7 @@
         <v>1087</v>
       </c>
     </row>
-    <row r="205" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="205" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A205" s="19">
         <v>204</v>
       </c>
@@ -10593,7 +10590,7 @@
         <v>1088</v>
       </c>
     </row>
-    <row r="206" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="206" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A206" s="19">
         <v>205</v>
       </c>
@@ -10625,7 +10622,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="207" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="207" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A207" s="19">
         <v>206</v>
       </c>
@@ -10657,7 +10654,7 @@
         <v>1090</v>
       </c>
     </row>
-    <row r="208" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="208" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A208" s="19">
         <v>207</v>
       </c>
@@ -10689,7 +10686,7 @@
         <v>1091</v>
       </c>
     </row>
-    <row r="209" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="209" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A209" s="19">
         <v>208</v>
       </c>
@@ -10721,7 +10718,7 @@
         <v>1092</v>
       </c>
     </row>
-    <row r="210" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="210" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A210" s="19">
         <v>209</v>
       </c>
@@ -10753,7 +10750,7 @@
         <v>1093</v>
       </c>
     </row>
-    <row r="211" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="211" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A211" s="19">
         <v>210</v>
       </c>
@@ -10785,7 +10782,7 @@
         <v>1094</v>
       </c>
     </row>
-    <row r="212" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="212" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A212" s="19">
         <v>211</v>
       </c>
@@ -10817,7 +10814,7 @@
         <v>1095</v>
       </c>
     </row>
-    <row r="213" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="213" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A213" s="19">
         <v>212</v>
       </c>
@@ -10849,7 +10846,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="214" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="214" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A214" s="19">
         <v>213</v>
       </c>
@@ -10881,7 +10878,7 @@
         <v>1097</v>
       </c>
     </row>
-    <row r="215" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="215" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A215" s="19">
         <v>214</v>
       </c>
@@ -10913,7 +10910,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="216" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="216" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A216" s="19">
         <v>215</v>
       </c>
@@ -10945,7 +10942,7 @@
         <v>1099</v>
       </c>
     </row>
-    <row r="217" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="217" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A217" s="19">
         <v>216</v>
       </c>
@@ -10977,7 +10974,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="218" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="218" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A218" s="19">
         <v>217</v>
       </c>
@@ -11009,7 +11006,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="219" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="219" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A219" s="19">
         <v>218</v>
       </c>
@@ -11041,7 +11038,7 @@
         <v>1102</v>
       </c>
     </row>
-    <row r="220" spans="1:10" ht="33.950000000000003" hidden="1" customHeight="1">
+    <row r="220" spans="1:10" ht="33.950000000000003" customHeight="1">
       <c r="A220" s="19">
         <v>219</v>
       </c>

</xml_diff>